<commit_message>
added neutrophil count & phospate, log variable selection
</commit_message>
<xml_diff>
--- a/preprocessing/geneva_stroke_unit_preprocessing/variable_assembly/selected_variables.xlsx
+++ b/preprocessing/geneva_stroke_unit_preprocessing/variable_assembly/selected_variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jk1/stroke_research/OPSUM/preprocessing/geneva_stroke_unit_preprocessing/variable_assembly/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{000B1AAA-97B4-D447-A533-67295FE8B088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F42D44-6846-834D-9C69-73D77271F34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{4EF3017B-64DF-5142-A0B6-DCCDE5805A97}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="19200" windowHeight="21000" xr2:uid="{4EF3017B-64DF-5142-A0B6-DCCDE5805A97}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>Activite anti-Xa (DOAC)</t>
   </si>
@@ -266,6 +266,12 @@
   </si>
   <si>
     <t>G-Sga-pH(T), ABL</t>
+  </si>
+  <si>
+    <t>neutrophiles-nb abs</t>
+  </si>
+  <si>
+    <t>phosphates</t>
   </si>
 </sst>
 </file>
@@ -634,7 +640,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E68269D3-7424-0349-8C48-DE37DFBA5500}">
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -984,6 +990,16 @@
         <v>63</v>
       </c>
     </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>78</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>